<commit_message>
added chrome report feature
</commit_message>
<xml_diff>
--- a/reports/report.xlsx
+++ b/reports/report.xlsx
@@ -445,7 +445,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>37.05161600001156</v>
+        <v>37.99269880005158</v>
       </c>
     </row>
     <row r="3">
@@ -460,7 +460,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>20.84180910000578</v>
+        <v>22.14527960005216</v>
       </c>
     </row>
     <row r="4">
@@ -475,7 +475,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>28.50361380004324</v>
+        <v>26.10934989992529</v>
       </c>
     </row>
     <row r="5">
@@ -490,7 +490,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>28.58569550001994</v>
+        <v>27.35174189996906</v>
       </c>
     </row>
     <row r="6">
@@ -505,7 +505,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>28.4995892001316</v>
+        <v>28.35954069998115</v>
       </c>
     </row>
     <row r="7">
@@ -520,7 +520,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>27.29184930003248</v>
+        <v>26.23254909995012</v>
       </c>
     </row>
     <row r="8">
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>26.88401550007984</v>
+        <v>28.20734920003451</v>
       </c>
     </row>
   </sheetData>

</xml_diff>